<commit_message>
Add transaction date, user-based toggle, Excel import for subscriptions
</commit_message>
<xml_diff>
--- a/dummy_subscriptions.xlsx
+++ b/dummy_subscriptions.xlsx
@@ -398,18 +398,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:K13"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
     <col min="3" max="3" width="28.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="8.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="28.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" customWidth="1"/>
     <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="35.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -417,30 +418,33 @@
         <v>ref</v>
       </c>
       <c r="B1" t="str">
+        <v>transaction_date</v>
+      </c>
+      <c r="C1" t="str">
         <v>customer_name</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>product_name</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>billing_period</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>price</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>payment_status</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>auto_renewal</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>is_user_based</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>start_date</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>notes</v>
       </c>
     </row>
@@ -449,30 +453,33 @@
         <v>S001</v>
       </c>
       <c r="B2" t="str">
+        <v>2021-03-28</v>
+      </c>
+      <c r="C2" t="str">
         <v>Vrushali Infotech Pvt Ltd</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>AMC Standard</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>yearly</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>6000</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>paid</v>
       </c>
-      <c r="G2" t="str">
-        <v>yes</v>
-      </c>
       <c r="H2" t="str">
+        <v>yes</v>
+      </c>
+      <c r="I2" t="str">
         <v>no</v>
       </c>
-      <c r="I2" t="str">
-        <v>2026-04-01</v>
-      </c>
       <c r="J2" t="str">
+        <v>2021-04-01</v>
+      </c>
+      <c r="K2" t="str">
         <v>AMC for 5 computers</v>
       </c>
     </row>
@@ -481,30 +488,33 @@
         <v>S002</v>
       </c>
       <c r="B3" t="str">
+        <v>2021-03-10</v>
+      </c>
+      <c r="C3" t="str">
         <v>Ganesh Traders</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>Domain Registration (.com)</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>yearly</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>1200</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>paid</v>
       </c>
-      <c r="G3" t="str">
-        <v>yes</v>
-      </c>
       <c r="H3" t="str">
+        <v>yes</v>
+      </c>
+      <c r="I3" t="str">
         <v>no</v>
       </c>
-      <c r="I3" t="str">
-        <v>2026-03-15</v>
-      </c>
       <c r="J3" t="str">
+        <v>2021-03-15</v>
+      </c>
+      <c r="K3" t="str">
         <v>Domain ganeshtraders.com</v>
       </c>
     </row>
@@ -513,30 +523,33 @@
         <v>S003</v>
       </c>
       <c r="B4" t="str">
+        <v>2022-04-25</v>
+      </c>
+      <c r="C4" t="str">
         <v>Shree Enterprises</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>Web Hosting Basic</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>yearly</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>2500</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>unpaid</v>
-      </c>
-      <c r="G4" t="str">
-        <v>no</v>
       </c>
       <c r="H4" t="str">
         <v>no</v>
       </c>
       <c r="I4" t="str">
-        <v>2026-05-01</v>
+        <v>no</v>
       </c>
       <c r="J4" t="str">
+        <v>2022-05-01</v>
+      </c>
+      <c r="K4" t="str">
         <v>cPanel hosting</v>
       </c>
     </row>
@@ -545,31 +558,34 @@
         <v>S004</v>
       </c>
       <c r="B5" t="str">
+        <v>2021-01-05</v>
+      </c>
+      <c r="C5" t="str">
         <v>Mahesh Auto Parts</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>AMC Premium</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>yearly</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>12000</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>paid</v>
       </c>
-      <c r="G5" t="str">
-        <v>yes</v>
-      </c>
       <c r="H5" t="str">
+        <v>yes</v>
+      </c>
+      <c r="I5" t="str">
         <v>no</v>
       </c>
-      <c r="I5" t="str">
-        <v>2026-01-10</v>
-      </c>
       <c r="J5" t="str">
-        <v>Priority AMC with on-site</v>
+        <v>2021-01-10</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Priority AMC</v>
       </c>
     </row>
     <row r="6">
@@ -577,31 +593,34 @@
         <v>S005</v>
       </c>
       <c r="B6" t="str">
+        <v>2023-05-28</v>
+      </c>
+      <c r="C6" t="str">
         <v>Krishna Agro</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
         <v>AMC Basic</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>yearly</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>3500</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>unpaid</v>
-      </c>
-      <c r="G6" t="str">
-        <v>no</v>
       </c>
       <c r="H6" t="str">
         <v>no</v>
       </c>
       <c r="I6" t="str">
-        <v>2026-06-01</v>
+        <v>no</v>
       </c>
       <c r="J6" t="str">
-        <v>Basic remote support only</v>
+        <v>2023-06-01</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Basic remote support</v>
       </c>
     </row>
     <row r="7">
@@ -609,30 +628,33 @@
         <v>S006</v>
       </c>
       <c r="B7" t="str">
+        <v>2021-03-25</v>
+      </c>
+      <c r="C7" t="str">
         <v>Pooja Consultancy</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
         <v>Tally Prime Single User</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>yearly</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <v>13500</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>paid</v>
       </c>
-      <c r="G7" t="str">
-        <v>yes</v>
-      </c>
       <c r="H7" t="str">
         <v>yes</v>
       </c>
       <c r="I7" t="str">
-        <v>2026-04-01</v>
+        <v>yes</v>
       </c>
       <c r="J7" t="str">
+        <v>2021-04-01</v>
+      </c>
+      <c r="K7" t="str">
         <v/>
       </c>
     </row>
@@ -641,30 +663,33 @@
         <v>S007</v>
       </c>
       <c r="B8" t="str">
+        <v>2022-01-28</v>
+      </c>
+      <c r="C8" t="str">
         <v>Sunita Medical Store</v>
       </c>
-      <c r="C8" t="str">
+      <c r="D8" t="str">
         <v>Busy Accounting Software</v>
       </c>
-      <c r="D8" t="str">
+      <c r="E8" t="str">
         <v>yearly</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <v>8500</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>paid</v>
       </c>
-      <c r="G8" t="str">
+      <c r="H8" t="str">
         <v>no</v>
       </c>
-      <c r="H8" t="str">
-        <v>yes</v>
-      </c>
       <c r="I8" t="str">
-        <v>2026-02-01</v>
+        <v>yes</v>
       </c>
       <c r="J8" t="str">
+        <v>2022-02-01</v>
+      </c>
+      <c r="K8" t="str">
         <v/>
       </c>
     </row>
@@ -673,31 +698,34 @@
         <v>S008</v>
       </c>
       <c r="B9" t="str">
+        <v>2023-05-10</v>
+      </c>
+      <c r="C9" t="str">
         <v>Deepak Hardware</v>
       </c>
-      <c r="C9" t="str">
+      <c r="D9" t="str">
         <v>GST Filing Software</v>
       </c>
-      <c r="D9" t="str">
+      <c r="E9" t="str">
         <v>yearly</v>
       </c>
-      <c r="E9" t="str">
+      <c r="F9" t="str">
         <v>4500</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v>unpaid</v>
       </c>
-      <c r="G9" t="str">
+      <c r="H9" t="str">
         <v>no</v>
       </c>
-      <c r="H9" t="str">
-        <v>yes</v>
-      </c>
       <c r="I9" t="str">
-        <v>2026-05-15</v>
+        <v>yes</v>
       </c>
       <c r="J9" t="str">
-        <v>Trial period started</v>
+        <v>2023-05-15</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Trial period</v>
       </c>
     </row>
     <row r="10">
@@ -705,30 +733,33 @@
         <v>S009</v>
       </c>
       <c r="B10" t="str">
+        <v>2022-03-28</v>
+      </c>
+      <c r="C10" t="str">
         <v>Vrushali Infotech Pvt Ltd</v>
       </c>
-      <c r="C10" t="str">
+      <c r="D10" t="str">
         <v>Tally Prime Multi User (5)</v>
       </c>
-      <c r="D10" t="str">
+      <c r="E10" t="str">
         <v>yearly</v>
       </c>
-      <c r="E10" t="str">
+      <c r="F10" t="str">
         <v>38000</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v>paid</v>
       </c>
-      <c r="G10" t="str">
-        <v>yes</v>
-      </c>
       <c r="H10" t="str">
         <v>yes</v>
       </c>
       <c r="I10" t="str">
-        <v>2026-04-01</v>
+        <v>yes</v>
       </c>
       <c r="J10" t="str">
+        <v>2022-04-01</v>
+      </c>
+      <c r="K10" t="str">
         <v>5 user license</v>
       </c>
     </row>
@@ -737,31 +768,34 @@
         <v>S010</v>
       </c>
       <c r="B11" t="str">
+        <v>2021-02-25</v>
+      </c>
+      <c r="C11" t="str">
         <v>Laxmi Finance</v>
       </c>
-      <c r="C11" t="str">
+      <c r="D11" t="str">
         <v>Tally Gold</v>
       </c>
-      <c r="D11" t="str">
+      <c r="E11" t="str">
         <v>yearly</v>
       </c>
-      <c r="E11" t="str">
+      <c r="F11" t="str">
         <v>25000</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>partial</v>
       </c>
-      <c r="G11" t="str">
-        <v>yes</v>
-      </c>
       <c r="H11" t="str">
         <v>yes</v>
       </c>
       <c r="I11" t="str">
-        <v>2026-03-01</v>
+        <v>yes</v>
       </c>
       <c r="J11" t="str">
-        <v>10 users Nashik office</v>
+        <v>2021-03-01</v>
+      </c>
+      <c r="K11" t="str">
+        <v>10 users Nashik</v>
       </c>
     </row>
     <row r="12">
@@ -769,30 +803,33 @@
         <v>S011</v>
       </c>
       <c r="B12" t="str">
+        <v>2020-12-28</v>
+      </c>
+      <c r="C12" t="str">
         <v>Amit Jewellers</v>
       </c>
-      <c r="C12" t="str">
+      <c r="D12" t="str">
         <v>Tally Prime Single User</v>
       </c>
-      <c r="D12" t="str">
+      <c r="E12" t="str">
         <v>yearly</v>
       </c>
-      <c r="E12" t="str">
+      <c r="F12" t="str">
         <v>13500</v>
       </c>
-      <c r="F12" t="str">
+      <c r="G12" t="str">
         <v>paid</v>
       </c>
-      <c r="G12" t="str">
-        <v>yes</v>
-      </c>
       <c r="H12" t="str">
         <v>yes</v>
       </c>
       <c r="I12" t="str">
-        <v>2026-01-01</v>
+        <v>yes</v>
       </c>
       <c r="J12" t="str">
+        <v>2021-01-01</v>
+      </c>
+      <c r="K12" t="str">
         <v>2 users showroom</v>
       </c>
     </row>
@@ -801,43 +838,46 @@
         <v>S012</v>
       </c>
       <c r="B13" t="str">
+        <v>2024-04-28</v>
+      </c>
+      <c r="C13" t="str">
         <v>Raj Constructions</v>
       </c>
-      <c r="C13" t="str">
+      <c r="D13" t="str">
         <v>Remote Desktop License</v>
       </c>
-      <c r="D13" t="str">
+      <c r="E13" t="str">
         <v>monthly</v>
       </c>
-      <c r="E13" t="str">
+      <c r="F13" t="str">
         <v>2000</v>
       </c>
-      <c r="F13" t="str">
+      <c r="G13" t="str">
         <v>unpaid</v>
       </c>
-      <c r="G13" t="str">
+      <c r="H13" t="str">
         <v>no</v>
       </c>
-      <c r="H13" t="str">
-        <v>yes</v>
-      </c>
       <c r="I13" t="str">
-        <v>2026-05-01</v>
+        <v>yes</v>
       </c>
       <c r="J13" t="str">
+        <v>2024-05-01</v>
+      </c>
+      <c r="K13" t="str">
         <v>3 remote users</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F20"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -875,16 +915,16 @@
         <v>Pooja Sharma</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-04-01</v>
+        <v>2021-04-01</v>
       </c>
       <c r="D2" t="str">
-        <v>2027-03-31</v>
+        <v>2022-03-31</v>
       </c>
       <c r="E2" t="str">
         <v>13500</v>
       </c>
       <c r="F2" t="str">
-        <v>Tally Prime - GST + Payroll module</v>
+        <v>Tally Prime - GST + Payroll</v>
       </c>
     </row>
     <row r="3">
@@ -895,16 +935,16 @@
         <v>Sunita Patil</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-02-01</v>
+        <v>2022-02-01</v>
       </c>
       <c r="D3" t="str">
-        <v>2027-01-31</v>
+        <v>2023-01-31</v>
       </c>
       <c r="E3" t="str">
         <v>8500</v>
       </c>
       <c r="F3" t="str">
-        <v>Busy software - medical billing</v>
+        <v>Busy - medical billing</v>
       </c>
     </row>
     <row r="4">
@@ -915,10 +955,10 @@
         <v>Deepak Joshi</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-05-15</v>
+        <v>2023-05-15</v>
       </c>
       <c r="D4" t="str">
-        <v>2027-05-14</v>
+        <v>2024-05-14</v>
       </c>
       <c r="E4" t="str">
         <v>4500</v>
@@ -935,16 +975,16 @@
         <v>Ganesh Chavan</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-04-01</v>
+        <v>2022-04-01</v>
       </c>
       <c r="D5" t="str">
-        <v>2027-03-31</v>
+        <v>2023-03-31</v>
       </c>
       <c r="E5" t="str">
         <v>8000</v>
       </c>
       <c r="F5" t="str">
-        <v>Admin user - full access</v>
+        <v>Admin - full access</v>
       </c>
     </row>
     <row r="6">
@@ -955,16 +995,16 @@
         <v>Priya Desai</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-04-01</v>
+        <v>2022-04-01</v>
       </c>
       <c r="D6" t="str">
-        <v>2027-03-31</v>
+        <v>2023-03-31</v>
       </c>
       <c r="E6" t="str">
         <v>7500</v>
       </c>
       <c r="F6" t="str">
-        <v>Accounts department</v>
+        <v>Accounts dept</v>
       </c>
     </row>
     <row r="7">
@@ -975,16 +1015,16 @@
         <v>Rahul Kulkarni</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-05-01</v>
+        <v>2022-05-01</v>
       </c>
       <c r="D7" t="str">
-        <v>2027-04-30</v>
+        <v>2023-04-30</v>
       </c>
       <c r="E7" t="str">
         <v>7500</v>
       </c>
       <c r="F7" t="str">
-        <v>Sales department - added later</v>
+        <v>Sales dept</v>
       </c>
     </row>
     <row r="8">
@@ -995,16 +1035,16 @@
         <v>Sneha More</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-06-01</v>
+        <v>2022-06-01</v>
       </c>
       <c r="D8" t="str">
-        <v>2027-05-31</v>
+        <v>2023-05-31</v>
       </c>
       <c r="E8" t="str">
         <v>7500</v>
       </c>
       <c r="F8" t="str">
-        <v>HR department - added June</v>
+        <v>HR dept</v>
       </c>
     </row>
     <row r="9">
@@ -1015,16 +1055,16 @@
         <v>Amit Pawar</v>
       </c>
       <c r="C9" t="str">
-        <v>2026-07-01</v>
+        <v>2022-07-01</v>
       </c>
       <c r="D9" t="str">
-        <v>2027-06-30</v>
+        <v>2023-06-30</v>
       </c>
       <c r="E9" t="str">
         <v>7500</v>
       </c>
       <c r="F9" t="str">
-        <v>Purchase department</v>
+        <v>Purchase dept</v>
       </c>
     </row>
     <row r="10">
@@ -1035,16 +1075,16 @@
         <v>Laxmi Patil</v>
       </c>
       <c r="C10" t="str">
-        <v>2026-03-01</v>
+        <v>2021-03-01</v>
       </c>
       <c r="D10" t="str">
-        <v>2027-02-28</v>
+        <v>2022-02-28</v>
       </c>
       <c r="E10" t="str">
         <v>3000</v>
       </c>
       <c r="F10" t="str">
-        <v>Owner - admin access</v>
+        <v>Owner - admin</v>
       </c>
     </row>
     <row r="11">
@@ -1055,10 +1095,10 @@
         <v>Suresh Nair</v>
       </c>
       <c r="C11" t="str">
-        <v>2026-03-01</v>
+        <v>2021-03-01</v>
       </c>
       <c r="D11" t="str">
-        <v>2027-02-28</v>
+        <v>2022-02-28</v>
       </c>
       <c r="E11" t="str">
         <v>2500</v>
@@ -1075,10 +1115,10 @@
         <v>Meena Shah</v>
       </c>
       <c r="C12" t="str">
-        <v>2026-03-01</v>
+        <v>2021-03-01</v>
       </c>
       <c r="D12" t="str">
-        <v>2027-02-28</v>
+        <v>2022-02-28</v>
       </c>
       <c r="E12" t="str">
         <v>2500</v>
@@ -1095,16 +1135,16 @@
         <v>Ravi Kumar</v>
       </c>
       <c r="C13" t="str">
-        <v>2026-04-01</v>
+        <v>2021-04-01</v>
       </c>
       <c r="D13" t="str">
-        <v>2027-03-31</v>
+        <v>2022-03-31</v>
       </c>
       <c r="E13" t="str">
         <v>2500</v>
       </c>
       <c r="F13" t="str">
-        <v>Loan department</v>
+        <v>Loan dept</v>
       </c>
     </row>
     <row r="14">
@@ -1115,16 +1155,16 @@
         <v>Anita Joshi</v>
       </c>
       <c r="C14" t="str">
-        <v>2026-04-01</v>
+        <v>2021-04-01</v>
       </c>
       <c r="D14" t="str">
-        <v>2027-03-31</v>
+        <v>2022-03-31</v>
       </c>
       <c r="E14" t="str">
         <v>2500</v>
       </c>
       <c r="F14" t="str">
-        <v>Recovery department</v>
+        <v>Recovery dept</v>
       </c>
     </row>
     <row r="15">
@@ -1135,201 +1175,121 @@
         <v>Vijay Tiwari</v>
       </c>
       <c r="C15" t="str">
-        <v>2026-05-01</v>
+        <v>2021-05-01</v>
       </c>
       <c r="D15" t="str">
-        <v>2027-04-30</v>
+        <v>2022-04-30</v>
       </c>
       <c r="E15" t="str">
         <v>2500</v>
       </c>
       <c r="F15" t="str">
-        <v>Branch manager Nashik</v>
+        <v>Branch manager</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>S010</v>
+        <v>S011</v>
       </c>
       <c r="B16" t="str">
-        <v>Pooja Rane</v>
+        <v>Amit Mehta</v>
       </c>
       <c r="C16" t="str">
-        <v>2026-06-01</v>
+        <v>2021-01-01</v>
       </c>
       <c r="D16" t="str">
-        <v>2027-05-31</v>
+        <v>2021-12-31</v>
       </c>
       <c r="E16" t="str">
-        <v>2500</v>
+        <v>7000</v>
       </c>
       <c r="F16" t="str">
-        <v>New joiner - June</v>
+        <v>Main showroom - owner</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>S010</v>
+        <v>S011</v>
       </c>
       <c r="B17" t="str">
-        <v>Kiran Wagh</v>
+        <v>Rekha Mehta</v>
       </c>
       <c r="C17" t="str">
-        <v>2026-07-01</v>
+        <v>2021-01-01</v>
       </c>
       <c r="D17" t="str">
-        <v>2027-06-30</v>
+        <v>2021-12-31</v>
       </c>
       <c r="E17" t="str">
-        <v>2500</v>
+        <v>6500</v>
       </c>
       <c r="F17" t="str">
-        <v>New joiner - July</v>
+        <v>Accounts</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>S010</v>
+        <v>S012</v>
       </c>
       <c r="B18" t="str">
-        <v>Nilesh Gaikwad</v>
+        <v>Rajesh Sharma</v>
       </c>
       <c r="C18" t="str">
-        <v>2026-08-01</v>
+        <v>2024-05-01</v>
       </c>
       <c r="D18" t="str">
-        <v>2027-07-31</v>
+        <v>2024-05-31</v>
       </c>
       <c r="E18" t="str">
-        <v>2500</v>
+        <v>700</v>
       </c>
       <c r="F18" t="str">
-        <v>Pending - Aug start</v>
+        <v>Site engineer</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>S010</v>
+        <v>S012</v>
       </c>
       <c r="B19" t="str">
-        <v>Sonal Bhosale</v>
+        <v>Sunil Patil</v>
       </c>
       <c r="C19" t="str">
-        <v>2026-09-01</v>
+        <v>2024-05-01</v>
       </c>
       <c r="D19" t="str">
-        <v>2027-08-31</v>
+        <v>2024-05-31</v>
       </c>
       <c r="E19" t="str">
-        <v>2500</v>
+        <v>700</v>
       </c>
       <c r="F19" t="str">
-        <v>Pending - Sep start</v>
+        <v>Office manager</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>S011</v>
+        <v>S012</v>
       </c>
       <c r="B20" t="str">
-        <v>Amit Mehta</v>
+        <v>Kavita Rao</v>
       </c>
       <c r="C20" t="str">
-        <v>2026-01-01</v>
+        <v>2024-06-01</v>
       </c>
       <c r="D20" t="str">
-        <v>2026-12-31</v>
+        <v>2024-06-30</v>
       </c>
       <c r="E20" t="str">
-        <v>7000</v>
+        <v>600</v>
       </c>
       <c r="F20" t="str">
-        <v>Main showroom - owner</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>S011</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Rekha Mehta</v>
-      </c>
-      <c r="C21" t="str">
-        <v>2026-01-01</v>
-      </c>
-      <c r="D21" t="str">
-        <v>2026-12-31</v>
-      </c>
-      <c r="E21" t="str">
-        <v>6500</v>
-      </c>
-      <c r="F21" t="str">
-        <v>Accounts - wife</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>S012</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Rajesh Sharma</v>
-      </c>
-      <c r="C22" t="str">
-        <v>2026-05-01</v>
-      </c>
-      <c r="D22" t="str">
-        <v>2026-05-31</v>
-      </c>
-      <c r="E22" t="str">
-        <v>700</v>
-      </c>
-      <c r="F22" t="str">
-        <v>Site engineer - remote</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>S012</v>
-      </c>
-      <c r="B23" t="str">
-        <v>Sunil Patil</v>
-      </c>
-      <c r="C23" t="str">
-        <v>2026-05-01</v>
-      </c>
-      <c r="D23" t="str">
-        <v>2026-05-31</v>
-      </c>
-      <c r="E23" t="str">
-        <v>700</v>
-      </c>
-      <c r="F23" t="str">
-        <v>Office manager</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>S012</v>
-      </c>
-      <c r="B24" t="str">
-        <v>Kavita Rao</v>
-      </c>
-      <c r="C24" t="str">
-        <v>2026-06-01</v>
-      </c>
-      <c r="D24" t="str">
-        <v>2026-06-30</v>
-      </c>
-      <c r="E24" t="str">
-        <v>600</v>
-      </c>
-      <c r="F24" t="str">
         <v>Added next month</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>